<commit_message>
chore: save local work before merging with remote dental-app repo
</commit_message>
<xml_diff>
--- a/selenium-tests/Test Results/Excel/Failed_Test_Cases.xlsx
+++ b/selenium-tests/Test Results/Excel/Failed_Test_Cases.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E1"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -416,27 +416,9 @@
         <v>Failure Reason</v>
       </c>
     </row>
-    <row r="2" xml:space="preserve">
-      <c r="A2" t="str">
-        <v>TC_WEB_AUTH_001</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Authentication</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Verify Live User Login Journey</v>
-      </c>
-      <c r="D2" t="str">
-        <v>6164ms</v>
-      </c>
-      <c r="E2" t="str" xml:space="preserve">
-        <v xml:space="preserve">unknown error: net::ERR_CONNECTION_REFUSED
-  (Session info: chrome=150.0.7871.186)</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>